<commit_message>
Update inventory and product images
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -1,261 +1,26 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <Application>Microsoft Excel</Application>
-  <DocSecurity>0</DocSecurity>
-  <ScaleCrop>false</ScaleCrop>
-  <HeadingPairs>
-    <vt:vector size="2" baseType="variant">
-      <vt:variant>
-        <vt:lpstr>Worksheets</vt:lpstr>
-      </vt:variant>
-      <vt:variant>
-        <vt:i4>1</vt:i4>
-      </vt:variant>
-    </vt:vector>
-  </HeadingPairs>
-  <TitlesOfParts>
-    <vt:vector size="1" baseType="lpstr">
-      <vt:lpstr>Sheet1</vt:lpstr>
-    </vt:vector>
-  </TitlesOfParts>
-  <LinksUpToDate>false</LinksUpToDate>
-  <SharedDoc>false</SharedDoc>
-  <HyperlinksChanged>false</HyperlinksChanged>
-  <AppVersion>16.0300</AppVersion>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gsaik\Downloads\Hot_wheels\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1B530EF-A6BC-4FC6-A0A8-5A1067F0C3AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="0"/>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <cp:lastModifiedBy>SAI KIRAN JAMPU</cp:lastModifiedBy>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-20T10:31:24Z</dcterms:modified>
-</cp:coreProperties>
-</file>
-
-<file path=xl\metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="10">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="1"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="2"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="3"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="4"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="5"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="6"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="7"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="8"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="9"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <valueMetadata count="10">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-    <bk>
-      <rc t="1" v="1"/>
-    </bk>
-    <bk>
-      <rc t="1" v="2"/>
-    </bk>
-    <bk>
-      <rc t="1" v="3"/>
-    </bk>
-    <bk>
-      <rc t="1" v="4"/>
-    </bk>
-    <bk>
-      <rc t="1" v="5"/>
-    </bk>
-    <bk>
-      <rc t="1" v="6"/>
-    </bk>
-    <bk>
-      <rc t="1" v="7"/>
-    </bk>
-    <bk>
-      <rc t="1" v="8"/>
-    </bk>
-    <bk>
-      <rc t="1" v="9"/>
-    </bk>
-  </valueMetadata>
-</metadata>
-</file>
-
-<file path=xl\richData\rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
-</file>
-
-<file path=xl\richData\rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="10">
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>1</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>2</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>3</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>4</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>5</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>6</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>7</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>8</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>9</v>
-    <v>5</v>
-  </rv>
-</rvData>
-</file>
-
-<file path=xl\richData\rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <s t="_localImage">
-    <k n="_rvRel:LocalImageIdentifier" t="i"/>
-    <k n="CalcOrigin" t="i"/>
-  </s>
-</rvStructures>
-</file>
-
-<file path=xl\richData\richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
-<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <rel r:id="rId1"/>
-  <rel r:id="rId2"/>
-  <rel r:id="rId3"/>
-  <rel r:id="rId4"/>
-  <rel r:id="rId5"/>
-  <rel r:id="rId6"/>
-  <rel r:id="rId7"/>
-  <rel r:id="rId8"/>
-  <rel r:id="rId9"/>
-  <rel r:id="rId10"/>
-</richValueRels>
-</file>
-
-<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="58">
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="68">
   <si>
     <t>id</t>
   </si>
@@ -429,11 +194,41 @@
   </si>
   <si>
     <t>Black and Red </t>
+  </si>
+  <si>
+    <t>porsche-911-gt3-rs.jpeg</t>
+  </si>
+  <si>
+    <t>bmw-e36-m3-race.jpeg</t>
+  </si>
+  <si>
+    <t>ferrai-458 challenge.jpeg</t>
+  </si>
+  <si>
+    <t>porsche- 911 carrera.jpeg</t>
+  </si>
+  <si>
+    <t>bmw-318.jpeg</t>
+  </si>
+  <si>
+    <t>toyato gr supra.jpeg</t>
+  </si>
+  <si>
+    <t>formula-1-2024-redbullformula-1-team-4.jpeg</t>
+  </si>
+  <si>
+    <t>mclaren- formula.jpeg</t>
+  </si>
+  <si>
+    <t>mclern 750 s.jpeg</t>
+  </si>
+  <si>
+    <t>lv super silot.jpeg</t>
   </si>
 </sst>
 </file>
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -476,10 +271,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -497,7 +291,22 @@
 </styleSheet>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+  <rel r:id="rId2"/>
+  <rel r:id="rId3"/>
+  <rel r:id="rId4"/>
+  <rel r:id="rId5"/>
+  <rel r:id="rId6"/>
+  <rel r:id="rId7"/>
+  <rel r:id="rId8"/>
+  <rel r:id="rId9"/>
+  <rel r:id="rId10"/>
+</richValueRels>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -817,43 +626,23 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sai Kiran Jampu\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B960DBF-0F84-4C89-9BC4-DE3D40D2738E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="0"/>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O29"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="40.625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.8984375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="89.125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="172.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.09765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.8984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="89.09765625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="172.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -900,8 +689,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2">
         <v>1001</v>
       </c>
       <c r="B2" t="s">
@@ -940,17 +729,15 @@
       <c r="M2" t="s">
         <v>18</v>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>porsche-911-gt3-rs.jpeg</t>
-        </is>
+      <c r="N2" t="s">
+        <v>58</v>
       </c>
       <c r="O2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3">
         <v>1002</v>
       </c>
       <c r="B3" t="s">
@@ -989,17 +776,15 @@
       <c r="M3" t="s">
         <v>18</v>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>bmw-e36-m3-race.jpeg</t>
-        </is>
+      <c r="N3" t="s">
+        <v>59</v>
       </c>
       <c r="O3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4">
         <v>1003</v>
       </c>
       <c r="B4" t="s">
@@ -1038,17 +823,15 @@
       <c r="M4" t="s">
         <v>18</v>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>ferrari-458-challenge.jpeg</t>
-        </is>
+      <c r="N4" t="s">
+        <v>60</v>
       </c>
       <c r="O4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5">
         <v>1004</v>
       </c>
       <c r="B5" t="s">
@@ -1087,17 +870,15 @@
       <c r="M5" t="b">
         <v>1</v>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>porsche-911-carrera-cabriolet.jpeg</t>
-        </is>
+      <c r="N5" t="s">
+        <v>61</v>
       </c>
       <c r="O5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6">
         <v>1005</v>
       </c>
       <c r="B6" t="s">
@@ -1136,17 +917,15 @@
       <c r="M6" t="b">
         <v>1</v>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>1995-bmw-318ti.jpeg</t>
-        </is>
+      <c r="N6" t="s">
+        <v>62</v>
       </c>
       <c r="O6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7">
         <v>1006</v>
       </c>
       <c r="B7" t="s">
@@ -1185,17 +964,15 @@
       <c r="M7" t="b">
         <v>1</v>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>2023-toyota-gr-supra.jpeg</t>
-        </is>
+      <c r="N7" t="s">
+        <v>63</v>
       </c>
       <c r="O7" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A8">
         <v>1007</v>
       </c>
       <c r="B8" t="s">
@@ -1234,17 +1011,15 @@
       <c r="M8" t="b">
         <v>1</v>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>formula-1-oracle-red-bull-racing-rb20-11.jpeg</t>
-        </is>
+      <c r="N8" t="s">
+        <v>64</v>
       </c>
       <c r="O8" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9">
         <v>1008</v>
       </c>
       <c r="B9" t="s">
@@ -1283,17 +1058,15 @@
       <c r="M9" t="b">
         <v>1</v>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>formula-1-2024-mclaren-formula-1-team-4.jpeg</t>
-        </is>
+      <c r="N9" t="s">
+        <v>65</v>
       </c>
       <c r="O9" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A10">
         <v>1009</v>
       </c>
       <c r="B10" t="s">
@@ -1332,17 +1105,15 @@
       <c r="M10" t="b">
         <v>1</v>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>mclaren-750s.jpeg</t>
-        </is>
+      <c r="N10" t="s">
+        <v>66</v>
       </c>
       <c r="O10" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A11">
         <v>1010</v>
       </c>
       <c r="B11" t="s">
@@ -1381,16 +1152,14 @@
       <c r="M11" t="b">
         <v>1</v>
       </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>lb-super-silhouette-nissan-s15-silvia.jpeg</t>
-        </is>
+      <c r="N11" t="s">
+        <v>67</v>
       </c>
       <c r="O11" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="29" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D29" t="s">
         <v>15</v>
       </c>

</xml_diff>